<commit_message>
Additional data for EPKT
</commit_message>
<xml_diff>
--- a/data/APT_BBOX.xlsx
+++ b/data/APT_BBOX.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\speeters\repos\airport-dashboard\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E635CD5-8C93-4875-84E2-2D11E72B4E7E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4E65154-37D3-4460-96AA-3DE8475EB75B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="26160" windowHeight="13470" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Monitored" sheetId="6" r:id="rId1"/>
@@ -19,7 +19,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">All!$A$1:$D$199</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Monitored!$A$1:$D$135</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Monitored!$A$1:$D$136</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'NO Monit.'!$A$1:$D$106</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1760" uniqueCount="738">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1764" uniqueCount="740">
   <si>
     <t>AIRPORT</t>
   </si>
@@ -2268,6 +2268,12 @@
   </si>
   <si>
     <t>41.58398308014017, 41.598667543454965, 41.615869180909215, 41.62003973073927</t>
+  </si>
+  <si>
+    <t>Katowice</t>
+  </si>
+  <si>
+    <t>19.045866,50.465865,19.117267,50.485856</t>
   </si>
 </sst>
 </file>
@@ -2335,7 +2341,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="13">
+  <borders count="14">
     <border>
       <left/>
       <right/>
@@ -2511,12 +2517,25 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF999999"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF999999"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF999999"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -2577,6 +2596,7 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" quotePrefix="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="13" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2858,7 +2878,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D135"/>
+  <dimension ref="A1:D136"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22.42578125" bestFit="1" customWidth="1"/>
@@ -3581,116 +3601,116 @@
         <v>601</v>
       </c>
     </row>
-    <row r="52" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A52" s="17" t="s">
+    <row r="52" spans="1:4" s="14" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A52" s="13" t="s">
         <v>91</v>
       </c>
-      <c r="B52" s="17" t="s">
+      <c r="B52" s="40" t="s">
+        <v>241</v>
+      </c>
+      <c r="C52" s="13" t="s">
+        <v>738</v>
+      </c>
+      <c r="D52" s="40" t="s">
+        <v>739</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A53" s="17" t="s">
+        <v>91</v>
+      </c>
+      <c r="B53" s="17" t="s">
         <v>90</v>
       </c>
-      <c r="C52" s="17" t="s">
+      <c r="C53" s="17" t="s">
         <v>92</v>
       </c>
-      <c r="D52" s="17" t="s">
+      <c r="D53" s="17" t="s">
         <v>469</v>
       </c>
     </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A53" s="15" t="s">
+    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A54" s="15" t="s">
         <v>94</v>
       </c>
-      <c r="B53" s="15" t="s">
+      <c r="B54" s="15" t="s">
         <v>93</v>
       </c>
-      <c r="C53" s="15" t="s">
+      <c r="C54" s="15" t="s">
         <v>95</v>
       </c>
-      <c r="D53" s="15" t="s">
+      <c r="D54" s="15" t="s">
         <v>628</v>
       </c>
     </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A54" s="6" t="s">
+    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A55" s="6" t="s">
         <v>94</v>
       </c>
-      <c r="B54" s="6" t="s">
+      <c r="B55" s="6" t="s">
         <v>96</v>
       </c>
-      <c r="C54" s="6" t="s">
+      <c r="C55" s="6" t="s">
         <v>97</v>
       </c>
-      <c r="D54" s="6" t="s">
+      <c r="D55" s="6" t="s">
         <v>471</v>
       </c>
     </row>
-    <row r="55" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A55" s="16" t="s">
+    <row r="56" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A56" s="16" t="s">
         <v>94</v>
       </c>
-      <c r="B55" s="16" t="s">
+      <c r="B56" s="16" t="s">
         <v>632</v>
       </c>
-      <c r="C55" s="16" t="s">
+      <c r="C56" s="16" t="s">
         <v>656</v>
       </c>
-      <c r="D55" s="16" t="s">
+      <c r="D56" s="16" t="s">
         <v>654</v>
-      </c>
-    </row>
-    <row r="56" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A56" s="18" t="s">
-        <v>99</v>
-      </c>
-      <c r="B56" s="18" t="s">
-        <v>98</v>
-      </c>
-      <c r="C56" s="18" t="s">
-        <v>100</v>
-      </c>
-      <c r="D56" s="18" t="s">
-        <v>472</v>
       </c>
     </row>
     <row r="57" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A57" s="18" t="s">
+        <v>99</v>
+      </c>
+      <c r="B57" s="18" t="s">
+        <v>98</v>
+      </c>
+      <c r="C57" s="18" t="s">
+        <v>100</v>
+      </c>
+      <c r="D57" s="18" t="s">
+        <v>472</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A58" s="18" t="s">
         <v>102</v>
       </c>
-      <c r="B57" s="18" t="s">
+      <c r="B58" s="18" t="s">
         <v>101</v>
       </c>
-      <c r="C57" s="18" t="s">
+      <c r="C58" s="18" t="s">
         <v>103</v>
       </c>
-      <c r="D57" s="18" t="s">
+      <c r="D58" s="18" t="s">
         <v>629</v>
       </c>
     </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A58" s="15" t="s">
+    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A59" s="15" t="s">
         <v>105</v>
       </c>
-      <c r="B58" s="15" t="s">
+      <c r="B59" s="15" t="s">
         <v>104</v>
       </c>
-      <c r="C58" s="15" t="s">
+      <c r="C59" s="15" t="s">
         <v>106</v>
       </c>
-      <c r="D58" s="15" t="s">
+      <c r="D59" s="15" t="s">
         <v>474</v>
-      </c>
-    </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A59" s="6" t="s">
-        <v>105</v>
-      </c>
-      <c r="B59" s="6" t="s">
-        <v>107</v>
-      </c>
-      <c r="C59" s="6" t="s">
-        <v>108</v>
-      </c>
-      <c r="D59" s="6" t="s">
-        <v>475</v>
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.25">
@@ -3698,13 +3718,13 @@
         <v>105</v>
       </c>
       <c r="B60" s="6" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="C60" s="6" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="D60" s="6" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.25">
@@ -3712,167 +3732,167 @@
         <v>105</v>
       </c>
       <c r="B61" s="6" t="s">
+        <v>109</v>
+      </c>
+      <c r="C61" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="D61" s="6" t="s">
+        <v>476</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A62" s="6" t="s">
+        <v>105</v>
+      </c>
+      <c r="B62" s="6" t="s">
         <v>111</v>
       </c>
-      <c r="C61" s="6" t="s">
+      <c r="C62" s="6" t="s">
         <v>112</v>
       </c>
-      <c r="D61" s="6" t="s">
+      <c r="D62" s="6" t="s">
         <v>477</v>
       </c>
     </row>
-    <row r="62" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A62" s="17" t="s">
+    <row r="63" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A63" s="17" t="s">
         <v>105</v>
       </c>
-      <c r="B62" s="17" t="s">
+      <c r="B63" s="17" t="s">
         <v>113</v>
       </c>
-      <c r="C62" s="17" t="s">
+      <c r="C63" s="17" t="s">
         <v>114</v>
       </c>
-      <c r="D62" s="17" t="s">
+      <c r="D63" s="17" t="s">
         <v>478</v>
       </c>
     </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A63" s="19" t="s">
+    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A64" s="19" t="s">
         <v>657</v>
       </c>
-      <c r="B63" s="19" t="s">
+      <c r="B64" s="19" t="s">
         <v>633</v>
       </c>
-      <c r="C63" s="19" t="s">
+      <c r="C64" s="19" t="s">
         <v>658</v>
       </c>
-      <c r="D63" s="19" t="s">
+      <c r="D64" s="19" t="s">
         <v>685</v>
       </c>
     </row>
-    <row r="64" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A64" s="16" t="s">
+    <row r="65" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A65" s="16" t="s">
         <v>657</v>
       </c>
-      <c r="B64" s="16" t="s">
+      <c r="B65" s="16" t="s">
         <v>634</v>
       </c>
-      <c r="C64" s="16" t="s">
+      <c r="C65" s="16" t="s">
         <v>659</v>
       </c>
-      <c r="D64" s="16" t="s">
+      <c r="D65" s="16" t="s">
         <v>686</v>
       </c>
     </row>
-    <row r="65" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A65" s="21" t="s">
+    <row r="66" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A66" s="21" t="s">
         <v>660</v>
       </c>
-      <c r="B65" s="21" t="s">
+      <c r="B66" s="21" t="s">
         <v>635</v>
       </c>
-      <c r="C65" s="21" t="s">
+      <c r="C66" s="21" t="s">
         <v>661</v>
       </c>
-      <c r="D65" s="21" t="s">
+      <c r="D66" s="21" t="s">
         <v>687</v>
       </c>
     </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A66" s="36" t="s">
+    <row r="67" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A67" s="36" t="s">
         <v>116</v>
       </c>
-      <c r="B66" s="36" t="s">
+      <c r="B67" s="36" t="s">
         <v>115</v>
       </c>
-      <c r="C66" s="36" t="s">
+      <c r="C67" s="36" t="s">
         <v>117</v>
       </c>
-      <c r="D66" s="36" t="s">
+      <c r="D67" s="36" t="s">
         <v>479</v>
       </c>
     </row>
-    <row r="67" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A67" s="34" t="s">
+    <row r="68" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A68" s="34" t="s">
         <v>116</v>
       </c>
-      <c r="B67" s="34" t="s">
+      <c r="B68" s="34" t="s">
         <v>704</v>
       </c>
-      <c r="C67" s="34" t="s">
+      <c r="C68" s="34" t="s">
         <v>705</v>
       </c>
-      <c r="D67" s="35" t="s">
+      <c r="D68" s="35" t="s">
         <v>703</v>
       </c>
     </row>
-    <row r="68" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A68" s="33" t="s">
+    <row r="69" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A69" s="33" t="s">
         <v>116</v>
       </c>
-      <c r="B68" s="33" t="s">
+      <c r="B69" s="33" t="s">
         <v>706</v>
       </c>
-      <c r="C68" s="33" t="s">
+      <c r="C69" s="33" t="s">
         <v>708</v>
       </c>
-      <c r="D68" s="14" t="s">
+      <c r="D69" s="14" t="s">
         <v>707</v>
-      </c>
-    </row>
-    <row r="69" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A69" s="18" t="s">
-        <v>119</v>
-      </c>
-      <c r="B69" s="18" t="s">
-        <v>118</v>
-      </c>
-      <c r="C69" s="18" t="s">
-        <v>120</v>
-      </c>
-      <c r="D69" s="18" t="s">
-        <v>480</v>
       </c>
     </row>
     <row r="70" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A70" s="18" t="s">
+        <v>119</v>
+      </c>
+      <c r="B70" s="18" t="s">
+        <v>118</v>
+      </c>
+      <c r="C70" s="18" t="s">
+        <v>120</v>
+      </c>
+      <c r="D70" s="18" t="s">
+        <v>480</v>
+      </c>
+    </row>
+    <row r="71" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A71" s="18" t="s">
         <v>122</v>
       </c>
-      <c r="B70" s="18" t="s">
+      <c r="B71" s="18" t="s">
         <v>121</v>
       </c>
-      <c r="C70" s="18" t="s">
+      <c r="C71" s="18" t="s">
         <v>123</v>
       </c>
-      <c r="D70" s="18" t="s">
+      <c r="D71" s="18" t="s">
         <v>481</v>
       </c>
     </row>
-    <row r="71" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A71" s="15" t="s">
+    <row r="72" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A72" s="15" t="s">
         <v>105</v>
       </c>
-      <c r="B71" s="15" t="s">
+      <c r="B72" s="15" t="s">
         <v>124</v>
       </c>
-      <c r="C71" s="15" t="s">
+      <c r="C72" s="15" t="s">
         <v>125</v>
       </c>
-      <c r="D71" s="15" t="s">
+      <c r="D72" s="15" t="s">
         <v>482</v>
-      </c>
-    </row>
-    <row r="72" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A72" s="6" t="s">
-        <v>105</v>
-      </c>
-      <c r="B72" s="6" t="s">
-        <v>126</v>
-      </c>
-      <c r="C72" s="6" t="s">
-        <v>127</v>
-      </c>
-      <c r="D72" s="6" t="s">
-        <v>483</v>
       </c>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.25">
@@ -3880,13 +3900,13 @@
         <v>105</v>
       </c>
       <c r="B73" s="6" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="C73" s="6" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="D73" s="6" t="s">
-        <v>484</v>
+        <v>483</v>
       </c>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.25">
@@ -3894,13 +3914,13 @@
         <v>105</v>
       </c>
       <c r="B74" s="6" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="C74" s="6" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="D74" s="6" t="s">
-        <v>485</v>
+        <v>484</v>
       </c>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.25">
@@ -3908,13 +3928,13 @@
         <v>105</v>
       </c>
       <c r="B75" s="6" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="C75" s="6" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="D75" s="6" t="s">
-        <v>486</v>
+        <v>485</v>
       </c>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.25">
@@ -3922,13 +3942,13 @@
         <v>105</v>
       </c>
       <c r="B76" s="6" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="C76" s="6" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="D76" s="6" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.25">
@@ -3936,13 +3956,13 @@
         <v>105</v>
       </c>
       <c r="B77" s="6" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="C77" s="6" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="D77" s="6" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.25">
@@ -3950,55 +3970,55 @@
         <v>105</v>
       </c>
       <c r="B78" s="6" t="s">
+        <v>136</v>
+      </c>
+      <c r="C78" s="6" t="s">
+        <v>137</v>
+      </c>
+      <c r="D78" s="6" t="s">
+        <v>488</v>
+      </c>
+    </row>
+    <row r="79" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A79" s="6" t="s">
+        <v>105</v>
+      </c>
+      <c r="B79" s="6" t="s">
         <v>138</v>
       </c>
-      <c r="C78" s="6" t="s">
+      <c r="C79" s="6" t="s">
         <v>139</v>
       </c>
-      <c r="D78" s="6" t="s">
+      <c r="D79" s="6" t="s">
         <v>489</v>
       </c>
     </row>
-    <row r="79" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A79" s="17" t="s">
+    <row r="80" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A80" s="17" t="s">
         <v>105</v>
       </c>
-      <c r="B79" s="17" t="s">
+      <c r="B80" s="17" t="s">
         <v>140</v>
       </c>
-      <c r="C79" s="17" t="s">
+      <c r="C80" s="17" t="s">
         <v>141</v>
       </c>
-      <c r="D79" s="17" t="s">
+      <c r="D80" s="17" t="s">
         <v>490</v>
       </c>
     </row>
-    <row r="80" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A80" s="20" t="s">
-        <v>143</v>
-      </c>
-      <c r="B80" s="20" t="s">
+    <row r="81" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A81" s="20" t="s">
+        <v>143</v>
+      </c>
+      <c r="B81" s="20" t="s">
         <v>281</v>
       </c>
-      <c r="C80" s="20" t="s">
+      <c r="C81" s="20" t="s">
         <v>282</v>
       </c>
-      <c r="D80" s="20" t="s">
+      <c r="D81" s="20" t="s">
         <v>537</v>
-      </c>
-    </row>
-    <row r="81" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A81" s="6" t="s">
-        <v>143</v>
-      </c>
-      <c r="B81" s="6" t="s">
-        <v>142</v>
-      </c>
-      <c r="C81" s="6" t="s">
-        <v>144</v>
-      </c>
-      <c r="D81" s="6" t="s">
-        <v>491</v>
       </c>
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.25">
@@ -4006,13 +4026,13 @@
         <v>143</v>
       </c>
       <c r="B82" s="6" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="C82" s="6" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="D82" s="6" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.25">
@@ -4020,13 +4040,13 @@
         <v>143</v>
       </c>
       <c r="B83" s="6" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="C83" s="6" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="D83" s="6" t="s">
-        <v>493</v>
+        <v>492</v>
       </c>
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.25">
@@ -4034,41 +4054,41 @@
         <v>143</v>
       </c>
       <c r="B84" s="6" t="s">
+        <v>147</v>
+      </c>
+      <c r="C84" s="6" t="s">
+        <v>148</v>
+      </c>
+      <c r="D84" s="6" t="s">
+        <v>493</v>
+      </c>
+    </row>
+    <row r="85" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A85" s="6" t="s">
+        <v>143</v>
+      </c>
+      <c r="B85" s="6" t="s">
         <v>149</v>
       </c>
-      <c r="C84" s="6" t="s">
+      <c r="C85" s="6" t="s">
         <v>150</v>
       </c>
-      <c r="D84" s="6" t="s">
+      <c r="D85" s="6" t="s">
         <v>494</v>
       </c>
     </row>
-    <row r="85" spans="1:4" s="14" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A85" s="13" t="s">
-        <v>143</v>
-      </c>
-      <c r="B85" s="13" t="s">
+    <row r="86" spans="1:4" s="14" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A86" s="13" t="s">
+        <v>143</v>
+      </c>
+      <c r="B86" s="13" t="s">
         <v>349</v>
       </c>
-      <c r="C85" s="13" t="s">
+      <c r="C86" s="13" t="s">
         <v>350</v>
       </c>
-      <c r="D85" s="13" t="s">
+      <c r="D86" s="13" t="s">
         <v>571</v>
-      </c>
-    </row>
-    <row r="86" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A86" s="6" t="s">
-        <v>143</v>
-      </c>
-      <c r="B86" s="6" t="s">
-        <v>151</v>
-      </c>
-      <c r="C86" s="6" t="s">
-        <v>152</v>
-      </c>
-      <c r="D86" s="6" t="s">
-        <v>495</v>
       </c>
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.25">
@@ -4076,69 +4096,69 @@
         <v>143</v>
       </c>
       <c r="B87" s="6" t="s">
+        <v>151</v>
+      </c>
+      <c r="C87" s="6" t="s">
+        <v>152</v>
+      </c>
+      <c r="D87" s="6" t="s">
+        <v>495</v>
+      </c>
+    </row>
+    <row r="88" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A88" s="6" t="s">
+        <v>143</v>
+      </c>
+      <c r="B88" s="6" t="s">
         <v>153</v>
       </c>
-      <c r="C87" s="6" t="s">
+      <c r="C88" s="6" t="s">
         <v>154</v>
       </c>
-      <c r="D87" s="6" t="s">
+      <c r="D88" s="6" t="s">
         <v>496</v>
       </c>
     </row>
-    <row r="88" spans="1:4" s="14" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A88" s="13" t="s">
-        <v>143</v>
-      </c>
-      <c r="B88" s="13" t="s">
+    <row r="89" spans="1:4" s="14" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A89" s="13" t="s">
+        <v>143</v>
+      </c>
+      <c r="B89" s="13" t="s">
         <v>371</v>
       </c>
-      <c r="C88" s="13" t="s">
+      <c r="C89" s="13" t="s">
         <v>372</v>
       </c>
-      <c r="D88" s="13" t="s">
+      <c r="D89" s="13" t="s">
         <v>582</v>
       </c>
     </row>
-    <row r="89" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A89" s="17" t="s">
-        <v>143</v>
-      </c>
-      <c r="B89" s="17" t="s">
+    <row r="90" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A90" s="17" t="s">
+        <v>143</v>
+      </c>
+      <c r="B90" s="17" t="s">
         <v>155</v>
       </c>
-      <c r="C89" s="17" t="s">
+      <c r="C90" s="17" t="s">
         <v>156</v>
       </c>
-      <c r="D89" s="17" t="s">
+      <c r="D90" s="17" t="s">
         <v>497</v>
       </c>
     </row>
-    <row r="90" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A90" s="15" t="s">
+    <row r="91" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A91" s="15" t="s">
         <v>158</v>
       </c>
-      <c r="B90" s="15" t="s">
+      <c r="B91" s="15" t="s">
         <v>157</v>
       </c>
-      <c r="C90" s="15" t="s">
+      <c r="C91" s="15" t="s">
         <v>159</v>
       </c>
-      <c r="D90" s="15" t="s">
+      <c r="D91" s="15" t="s">
         <v>498</v>
-      </c>
-    </row>
-    <row r="91" spans="1:4" s="14" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A91" s="13" t="s">
-        <v>158</v>
-      </c>
-      <c r="B91" s="13" t="s">
-        <v>636</v>
-      </c>
-      <c r="C91" s="13" t="s">
-        <v>662</v>
-      </c>
-      <c r="D91" s="13" t="s">
-        <v>688</v>
       </c>
     </row>
     <row r="92" spans="1:4" s="14" customFormat="1" x14ac:dyDescent="0.25">
@@ -4146,97 +4166,97 @@
         <v>158</v>
       </c>
       <c r="B92" s="13" t="s">
+        <v>636</v>
+      </c>
+      <c r="C92" s="13" t="s">
+        <v>662</v>
+      </c>
+      <c r="D92" s="13" t="s">
+        <v>688</v>
+      </c>
+    </row>
+    <row r="93" spans="1:4" s="14" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A93" s="13" t="s">
+        <v>158</v>
+      </c>
+      <c r="B93" s="13" t="s">
         <v>719</v>
       </c>
-      <c r="C92" s="13" t="s">
+      <c r="C93" s="13" t="s">
         <v>720</v>
       </c>
-      <c r="D92" s="13" t="s">
+      <c r="D93" s="13" t="s">
         <v>721</v>
       </c>
     </row>
-    <row r="93" spans="1:4" s="14" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A93" s="16" t="s">
+    <row r="94" spans="1:4" s="14" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A94" s="16" t="s">
         <v>158</v>
       </c>
-      <c r="B93" s="16" t="s">
+      <c r="B94" s="16" t="s">
         <v>637</v>
       </c>
-      <c r="C93" s="16" t="s">
+      <c r="C94" s="16" t="s">
         <v>663</v>
       </c>
-      <c r="D93" s="16" t="s">
+      <c r="D94" s="16" t="s">
         <v>689</v>
       </c>
     </row>
-    <row r="94" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A94" s="18" t="s">
+    <row r="95" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A95" s="18" t="s">
         <v>161</v>
       </c>
-      <c r="B94" s="18" t="s">
+      <c r="B95" s="18" t="s">
         <v>160</v>
       </c>
-      <c r="C94" s="18" t="s">
+      <c r="C95" s="18" t="s">
         <v>162</v>
       </c>
-      <c r="D94" s="18" t="s">
+      <c r="D95" s="18" t="s">
         <v>499</v>
       </c>
     </row>
-    <row r="95" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A95" s="15" t="s">
+    <row r="96" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A96" s="15" t="s">
         <v>164</v>
       </c>
-      <c r="B95" s="15" t="s">
+      <c r="B96" s="15" t="s">
         <v>723</v>
       </c>
-      <c r="C95" s="15" t="s">
+      <c r="C96" s="15" t="s">
         <v>722</v>
       </c>
-      <c r="D95" s="15" t="s">
+      <c r="D96" s="15" t="s">
         <v>727</v>
       </c>
     </row>
-    <row r="96" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A96" s="22" t="s">
+    <row r="97" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A97" s="22" t="s">
         <v>164</v>
       </c>
-      <c r="B96" s="22" t="s">
+      <c r="B97" s="22" t="s">
         <v>163</v>
       </c>
-      <c r="C96" s="22" t="s">
+      <c r="C97" s="22" t="s">
         <v>165</v>
       </c>
-      <c r="D96" s="22" t="s">
+      <c r="D97" s="22" t="s">
         <v>500</v>
       </c>
     </row>
-    <row r="97" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A97" s="13" t="s">
+    <row r="98" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A98" s="13" t="s">
         <v>164</v>
       </c>
-      <c r="B97" s="13" t="s">
+      <c r="B98" s="13" t="s">
         <v>638</v>
       </c>
-      <c r="C97" s="13" t="s">
+      <c r="C98" s="13" t="s">
         <v>664</v>
       </c>
-      <c r="D97" s="13" t="s">
+      <c r="D98" s="13" t="s">
         <v>690</v>
-      </c>
-    </row>
-    <row r="98" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A98" s="6" t="s">
-        <v>164</v>
-      </c>
-      <c r="B98" s="6" t="s">
-        <v>724</v>
-      </c>
-      <c r="C98" s="6" t="s">
-        <v>725</v>
-      </c>
-      <c r="D98" s="6" t="s">
-        <v>726</v>
       </c>
     </row>
     <row r="99" spans="1:4" x14ac:dyDescent="0.25">
@@ -4244,13 +4264,13 @@
         <v>164</v>
       </c>
       <c r="B99" s="6" t="s">
-        <v>166</v>
+        <v>724</v>
       </c>
       <c r="C99" s="6" t="s">
-        <v>167</v>
+        <v>725</v>
       </c>
       <c r="D99" s="6" t="s">
-        <v>502</v>
+        <v>726</v>
       </c>
     </row>
     <row r="100" spans="1:4" x14ac:dyDescent="0.25">
@@ -4258,13 +4278,13 @@
         <v>164</v>
       </c>
       <c r="B100" s="6" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="C100" s="6" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="D100" s="6" t="s">
-        <v>503</v>
+        <v>502</v>
       </c>
     </row>
     <row r="101" spans="1:4" x14ac:dyDescent="0.25">
@@ -4272,13 +4292,13 @@
         <v>164</v>
       </c>
       <c r="B101" s="6" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="C101" s="6" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="D101" s="6" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
     </row>
     <row r="102" spans="1:4" x14ac:dyDescent="0.25">
@@ -4286,13 +4306,13 @@
         <v>164</v>
       </c>
       <c r="B102" s="6" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="C102" s="6" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="D102" s="6" t="s">
-        <v>501</v>
+        <v>504</v>
       </c>
     </row>
     <row r="103" spans="1:4" x14ac:dyDescent="0.25">
@@ -4300,13 +4320,13 @@
         <v>164</v>
       </c>
       <c r="B103" s="6" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="C103" s="6" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="D103" s="6" t="s">
-        <v>505</v>
+        <v>501</v>
       </c>
     </row>
     <row r="104" spans="1:4" x14ac:dyDescent="0.25">
@@ -4314,27 +4334,27 @@
         <v>164</v>
       </c>
       <c r="B104" s="6" t="s">
+        <v>174</v>
+      </c>
+      <c r="C104" s="6" t="s">
+        <v>175</v>
+      </c>
+      <c r="D104" s="6" t="s">
+        <v>505</v>
+      </c>
+    </row>
+    <row r="105" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A105" s="6" t="s">
+        <v>164</v>
+      </c>
+      <c r="B105" s="6" t="s">
         <v>176</v>
       </c>
-      <c r="C104" s="6" t="s">
+      <c r="C105" s="6" t="s">
         <v>177</v>
       </c>
-      <c r="D104" s="6" t="s">
+      <c r="D105" s="6" t="s">
         <v>506</v>
-      </c>
-    </row>
-    <row r="105" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A105" s="12" t="s">
-        <v>164</v>
-      </c>
-      <c r="B105" s="12" t="s">
-        <v>178</v>
-      </c>
-      <c r="C105" s="12" t="s">
-        <v>179</v>
-      </c>
-      <c r="D105" s="12" t="s">
-        <v>508</v>
       </c>
     </row>
     <row r="106" spans="1:4" x14ac:dyDescent="0.25">
@@ -4342,223 +4362,223 @@
         <v>164</v>
       </c>
       <c r="B106" s="12" t="s">
+        <v>178</v>
+      </c>
+      <c r="C106" s="12" t="s">
+        <v>179</v>
+      </c>
+      <c r="D106" s="12" t="s">
+        <v>508</v>
+      </c>
+    </row>
+    <row r="107" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A107" s="12" t="s">
+        <v>164</v>
+      </c>
+      <c r="B107" s="12" t="s">
         <v>180</v>
       </c>
-      <c r="C106" s="12" t="s">
+      <c r="C107" s="12" t="s">
         <v>181</v>
       </c>
-      <c r="D106" s="12" t="s">
+      <c r="D107" s="12" t="s">
         <v>507</v>
       </c>
     </row>
-    <row r="107" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A107" s="24" t="s">
+    <row r="108" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A108" s="24" t="s">
         <v>164</v>
       </c>
-      <c r="B107" s="24" t="s">
+      <c r="B108" s="24" t="s">
         <v>182</v>
       </c>
-      <c r="C107" s="24" t="s">
+      <c r="C108" s="24" t="s">
         <v>183</v>
       </c>
-      <c r="D107" s="24" t="s">
+      <c r="D108" s="24" t="s">
         <v>509</v>
-      </c>
-    </row>
-    <row r="108" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A108" s="25" t="s">
-        <v>185</v>
-      </c>
-      <c r="B108" s="25" t="s">
-        <v>184</v>
-      </c>
-      <c r="C108" s="25" t="s">
-        <v>186</v>
-      </c>
-      <c r="D108" s="25" t="s">
-        <v>510</v>
       </c>
     </row>
     <row r="109" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A109" s="25" t="s">
+        <v>185</v>
+      </c>
+      <c r="B109" s="25" t="s">
+        <v>184</v>
+      </c>
+      <c r="C109" s="25" t="s">
+        <v>186</v>
+      </c>
+      <c r="D109" s="25" t="s">
+        <v>510</v>
+      </c>
+    </row>
+    <row r="110" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A110" s="25" t="s">
         <v>188</v>
       </c>
-      <c r="B109" s="25" t="s">
+      <c r="B110" s="25" t="s">
         <v>187</v>
       </c>
-      <c r="C109" s="25" t="s">
+      <c r="C110" s="25" t="s">
         <v>189</v>
       </c>
-      <c r="D109" s="25" t="s">
+      <c r="D110" s="25" t="s">
         <v>511</v>
       </c>
     </row>
-    <row r="110" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A110" s="27" t="s">
+    <row r="111" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A111" s="27" t="s">
         <v>665</v>
       </c>
-      <c r="B110" s="27" t="s">
+      <c r="B111" s="27" t="s">
         <v>639</v>
       </c>
-      <c r="C110" s="27" t="s">
+      <c r="C111" s="27" t="s">
         <v>666</v>
       </c>
-      <c r="D110" s="27" t="s">
+      <c r="D111" s="27" t="s">
         <v>691</v>
-      </c>
-    </row>
-    <row r="111" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A111" s="25" t="s">
-        <v>191</v>
-      </c>
-      <c r="B111" s="25" t="s">
-        <v>190</v>
-      </c>
-      <c r="C111" s="25" t="s">
-        <v>191</v>
-      </c>
-      <c r="D111" s="25" t="s">
-        <v>512</v>
       </c>
     </row>
     <row r="112" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A112" s="25" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="B112" s="25" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="C112" s="25" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="D112" s="25" t="s">
-        <v>513</v>
+        <v>512</v>
       </c>
     </row>
     <row r="113" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A113" s="25" t="s">
+        <v>193</v>
+      </c>
+      <c r="B113" s="25" t="s">
+        <v>192</v>
+      </c>
+      <c r="C113" s="25" t="s">
+        <v>194</v>
+      </c>
+      <c r="D113" s="25" t="s">
+        <v>513</v>
+      </c>
+    </row>
+    <row r="114" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A114" s="25" t="s">
         <v>196</v>
       </c>
-      <c r="B113" s="25" t="s">
+      <c r="B114" s="25" t="s">
         <v>213</v>
       </c>
-      <c r="C113" s="25" t="s">
+      <c r="C114" s="25" t="s">
         <v>214</v>
       </c>
-      <c r="D113" s="25" t="s">
+      <c r="D114" s="25" t="s">
         <v>521</v>
       </c>
     </row>
-    <row r="114" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A114" s="23" t="s">
+    <row r="115" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A115" s="23" t="s">
         <v>196</v>
       </c>
-      <c r="B114" s="23" t="s">
+      <c r="B115" s="23" t="s">
         <v>195</v>
       </c>
-      <c r="C114" s="23" t="s">
+      <c r="C115" s="23" t="s">
         <v>197</v>
       </c>
-      <c r="D114" s="23" t="s">
+      <c r="D115" s="23" t="s">
         <v>514</v>
       </c>
     </row>
-    <row r="115" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A115" s="12" t="s">
+    <row r="116" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A116" s="12" t="s">
         <v>196</v>
       </c>
-      <c r="B115" s="12" t="s">
+      <c r="B116" s="12" t="s">
         <v>198</v>
       </c>
-      <c r="C115" s="12" t="s">
+      <c r="C116" s="12" t="s">
         <v>199</v>
       </c>
-      <c r="D115" s="12" t="s">
+      <c r="D116" s="12" t="s">
         <v>515</v>
       </c>
     </row>
-    <row r="116" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A116" s="28" t="s">
+    <row r="117" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A117" s="28" t="s">
         <v>667</v>
       </c>
-      <c r="B116" s="28" t="s">
+      <c r="B117" s="28" t="s">
         <v>640</v>
       </c>
-      <c r="C116" s="28" t="s">
+      <c r="C117" s="28" t="s">
         <v>668</v>
       </c>
-      <c r="D116" s="28" t="s">
+      <c r="D117" s="28" t="s">
         <v>692</v>
       </c>
     </row>
-    <row r="117" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A117" s="25" t="s">
+    <row r="118" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A118" s="25" t="s">
         <v>201</v>
       </c>
-      <c r="B117" s="25" t="s">
+      <c r="B118" s="25" t="s">
         <v>200</v>
       </c>
-      <c r="C117" s="25" t="s">
+      <c r="C118" s="25" t="s">
         <v>202</v>
       </c>
-      <c r="D117" s="25" t="s">
+      <c r="D118" s="25" t="s">
         <v>516</v>
       </c>
     </row>
-    <row r="118" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A118" s="29" t="s">
+    <row r="119" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A119" s="29" t="s">
         <v>204</v>
       </c>
-      <c r="B118" s="29" t="s">
+      <c r="B119" s="29" t="s">
         <v>203</v>
       </c>
-      <c r="C118" s="29" t="s">
+      <c r="C119" s="29" t="s">
         <v>205</v>
       </c>
-      <c r="D118" s="29" t="s">
+      <c r="D119" s="29" t="s">
         <v>518</v>
       </c>
     </row>
-    <row r="119" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A119" s="30" t="s">
+    <row r="120" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A120" s="30" t="s">
         <v>204</v>
       </c>
-      <c r="B119" s="30" t="s">
+      <c r="B120" s="30" t="s">
         <v>206</v>
       </c>
-      <c r="C119" s="30" t="s">
+      <c r="C120" s="30" t="s">
         <v>207</v>
       </c>
-      <c r="D119" s="30" t="s">
+      <c r="D120" s="30" t="s">
         <v>517</v>
       </c>
     </row>
-    <row r="120" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A120" s="26" t="s">
+    <row r="121" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A121" s="26" t="s">
         <v>421</v>
       </c>
-      <c r="B120" s="26" t="s">
+      <c r="B121" s="26" t="s">
         <v>641</v>
       </c>
-      <c r="C120" s="26" t="s">
+      <c r="C121" s="26" t="s">
         <v>669</v>
       </c>
-      <c r="D120" s="26" t="s">
+      <c r="D121" s="26" t="s">
         <v>693</v>
-      </c>
-    </row>
-    <row r="121" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A121" s="31" t="s">
-        <v>421</v>
-      </c>
-      <c r="B121" s="31" t="s">
-        <v>422</v>
-      </c>
-      <c r="C121" s="31" t="s">
-        <v>423</v>
-      </c>
-      <c r="D121" s="31" t="s">
-        <v>625</v>
       </c>
     </row>
     <row r="122" spans="1:4" x14ac:dyDescent="0.25">
@@ -4566,13 +4586,13 @@
         <v>421</v>
       </c>
       <c r="B122" s="31" t="s">
-        <v>424</v>
+        <v>422</v>
       </c>
       <c r="C122" s="31" t="s">
-        <v>425</v>
+        <v>423</v>
       </c>
       <c r="D122" s="31" t="s">
-        <v>626</v>
+        <v>625</v>
       </c>
     </row>
     <row r="123" spans="1:4" x14ac:dyDescent="0.25">
@@ -4580,13 +4600,13 @@
         <v>421</v>
       </c>
       <c r="B123" s="31" t="s">
-        <v>642</v>
+        <v>424</v>
       </c>
       <c r="C123" s="31" t="s">
-        <v>670</v>
+        <v>425</v>
       </c>
       <c r="D123" s="31" t="s">
-        <v>694</v>
+        <v>626</v>
       </c>
     </row>
     <row r="124" spans="1:4" x14ac:dyDescent="0.25">
@@ -4594,173 +4614,187 @@
         <v>421</v>
       </c>
       <c r="B124" s="31" t="s">
+        <v>642</v>
+      </c>
+      <c r="C124" s="31" t="s">
+        <v>670</v>
+      </c>
+      <c r="D124" s="31" t="s">
+        <v>694</v>
+      </c>
+    </row>
+    <row r="125" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A125" s="31" t="s">
+        <v>421</v>
+      </c>
+      <c r="B125" s="31" t="s">
         <v>426</v>
       </c>
-      <c r="C124" s="31" t="s">
+      <c r="C125" s="31" t="s">
         <v>427</v>
       </c>
-      <c r="D124" s="31" t="s">
+      <c r="D125" s="31" t="s">
         <v>627</v>
       </c>
     </row>
-    <row r="125" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A125" s="32" t="s">
+    <row r="126" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A126" s="32" t="s">
         <v>421</v>
       </c>
-      <c r="B125" s="32" t="s">
+      <c r="B126" s="32" t="s">
         <v>643</v>
       </c>
-      <c r="C125" s="32" t="s">
+      <c r="C126" s="32" t="s">
         <v>671</v>
       </c>
-      <c r="D125" s="32" t="s">
+      <c r="D126" s="32" t="s">
         <v>701</v>
-      </c>
-    </row>
-    <row r="126" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A126" s="27" t="s">
-        <v>672</v>
-      </c>
-      <c r="B126" s="27" t="s">
-        <v>644</v>
-      </c>
-      <c r="C126" s="27" t="s">
-        <v>673</v>
-      </c>
-      <c r="D126" s="27" t="s">
-        <v>695</v>
       </c>
     </row>
     <row r="127" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A127" s="27" t="s">
+        <v>672</v>
+      </c>
+      <c r="B127" s="27" t="s">
+        <v>644</v>
+      </c>
+      <c r="C127" s="27" t="s">
+        <v>673</v>
+      </c>
+      <c r="D127" s="27" t="s">
+        <v>695</v>
+      </c>
+    </row>
+    <row r="128" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A128" s="27" t="s">
         <v>674</v>
       </c>
-      <c r="B127" s="27" t="s">
+      <c r="B128" s="27" t="s">
         <v>645</v>
       </c>
-      <c r="C127" s="27" t="s">
+      <c r="C128" s="27" t="s">
         <v>675</v>
       </c>
-      <c r="D127" s="27" t="s">
+      <c r="D128" s="27" t="s">
         <v>696</v>
       </c>
     </row>
-    <row r="128" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A128" s="26" t="s">
+    <row r="129" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A129" s="26" t="s">
         <v>676</v>
       </c>
-      <c r="B128" s="26" t="s">
+      <c r="B129" s="26" t="s">
         <v>646</v>
       </c>
-      <c r="C128" s="26" t="s">
+      <c r="C129" s="26" t="s">
         <v>677</v>
       </c>
-      <c r="D128" s="26" t="s">
+      <c r="D129" s="26" t="s">
         <v>697</v>
       </c>
     </row>
-    <row r="129" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A129" s="32" t="s">
+    <row r="130" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A130" s="32" t="s">
         <v>676</v>
       </c>
-      <c r="B129" s="32" t="s">
+      <c r="B130" s="32" t="s">
         <v>647</v>
       </c>
-      <c r="C129" s="32" t="s">
+      <c r="C130" s="32" t="s">
         <v>678</v>
       </c>
-      <c r="D129" s="32" t="s">
+      <c r="D130" s="32" t="s">
         <v>702</v>
       </c>
     </row>
-    <row r="130" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A130" s="25" t="s">
+    <row r="131" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A131" s="25" t="s">
         <v>209</v>
       </c>
-      <c r="B130" s="25" t="s">
+      <c r="B131" s="25" t="s">
         <v>208</v>
       </c>
-      <c r="C130" s="25" t="s">
+      <c r="C131" s="25" t="s">
         <v>210</v>
       </c>
-      <c r="D130" s="25" t="s">
+      <c r="D131" s="25" t="s">
         <v>519</v>
       </c>
     </row>
-    <row r="131" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A131" s="27" t="s">
+    <row r="132" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A132" s="27" t="s">
         <v>679</v>
       </c>
-      <c r="B131" s="27" t="s">
+      <c r="B132" s="27" t="s">
         <v>648</v>
       </c>
-      <c r="C131" s="27" t="s">
+      <c r="C132" s="27" t="s">
         <v>680</v>
       </c>
-      <c r="D131" s="27" t="s">
+      <c r="D132" s="27" t="s">
         <v>698</v>
-      </c>
-    </row>
-    <row r="132" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A132" s="39" t="s">
-        <v>681</v>
-      </c>
-      <c r="B132" s="39" t="s">
-        <v>649</v>
-      </c>
-      <c r="C132" s="39" t="s">
-        <v>682</v>
-      </c>
-      <c r="D132" s="39" t="s">
-        <v>699</v>
       </c>
     </row>
     <row r="133" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A133" s="39" t="s">
         <v>681</v>
       </c>
-      <c r="B133" s="31" t="s">
-        <v>732</v>
-      </c>
-      <c r="C133" t="s">
-        <v>734</v>
-      </c>
-      <c r="D133" s="31" t="s">
-        <v>736</v>
-      </c>
-    </row>
-    <row r="134" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B133" s="39" t="s">
+        <v>649</v>
+      </c>
+      <c r="C133" s="39" t="s">
+        <v>682</v>
+      </c>
+      <c r="D133" s="39" t="s">
+        <v>699</v>
+      </c>
+    </row>
+    <row r="134" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A134" s="39" t="s">
         <v>681</v>
       </c>
       <c r="B134" s="31" t="s">
+        <v>732</v>
+      </c>
+      <c r="C134" t="s">
+        <v>734</v>
+      </c>
+      <c r="D134" s="31" t="s">
+        <v>736</v>
+      </c>
+    </row>
+    <row r="135" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A135" s="39" t="s">
+        <v>681</v>
+      </c>
+      <c r="B135" s="31" t="s">
         <v>733</v>
       </c>
-      <c r="C134" t="s">
+      <c r="C135" t="s">
         <v>735</v>
       </c>
-      <c r="D134" s="31" t="s">
+      <c r="D135" s="31" t="s">
         <v>737</v>
       </c>
     </row>
-    <row r="135" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A135" s="27" t="s">
+    <row r="136" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A136" s="27" t="s">
         <v>683</v>
       </c>
-      <c r="B135" s="27" t="s">
+      <c r="B136" s="27" t="s">
         <v>650</v>
       </c>
-      <c r="C135" s="27" t="s">
+      <c r="C136" s="27" t="s">
         <v>684</v>
       </c>
-      <c r="D135" s="27" t="s">
+      <c r="D136" s="27" t="s">
         <v>700</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D135" xr:uid="{00000000-0009-0000-0000-000000000000}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D135">
-      <sortCondition ref="B1:B135"/>
+  <autoFilter ref="A1:D136" xr:uid="{00000000-0009-0000-0000-000000000000}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D136">
+      <sortCondition ref="B1:B136"/>
     </sortState>
   </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -9082,6 +9116,21 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101002D0FE5D67A8955468C14E1CD507D7C7A" ma:contentTypeVersion="0" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="c2136fc4bded2217ef16a7f65bc2a169">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="c64490b4aec6201516c3a874156f37b2">
     <xsd:element name="properties">
@@ -9195,33 +9244,10 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E59517FD-2FEA-4C30-82FF-FAEC56890ACA}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{01A91219-5C2C-423A-833B-AB294380AD1F}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -9242,9 +9268,17 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{01A91219-5C2C-423A-833B-AB294380AD1F}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E59517FD-2FEA-4C30-82FF-FAEC56890ACA}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>